<commit_message>
Refactor API: remove flags and split endpoints per comparison type
</commit_message>
<xml_diff>
--- a/output/table_differences.xlsx
+++ b/output/table_differences.xlsx
@@ -12,9 +12,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
-  <si>
-    <t>Table Differences: db1 vs db2</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="35">
+  <si>
+    <t>Table Differences: d1 vs d2</t>
   </si>
   <si>
     <t>#</t>
@@ -29,28 +29,94 @@
     <t>1</t>
   </si>
   <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>d1 &amp; d2</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>current_dept_emp</t>
+  </si>
+  <si>
+    <t>d1 only</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>department</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>dept_emp</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>dept_emp_latest_date</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>dept_manager</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
     <t>employee</t>
   </si>
   <si>
-    <t>db1 &amp; db2</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>orders</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>products</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>users</t>
+    <t>8</t>
+  </si>
+  <si>
+    <t>project</t>
+  </si>
+  <si>
+    <t>d2 only</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>region</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>region_emp</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>salary</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>salary_group</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>sg_emp</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>titles</t>
   </si>
 </sst>
 </file>
@@ -179,12 +245,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="6.09765625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="12.6875" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="13.578125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="6.90625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="22.66015625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="11.38671875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1" ht="20.0" customHeight="true">
@@ -221,16 +287,16 @@
       <c r="B4" t="s" s="7">
         <v>8</v>
       </c>
-      <c r="C4" t="s" s="3">
-        <v>6</v>
+      <c r="C4" t="s" s="4">
+        <v>9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="6">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s" s="6">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s" s="3">
         <v>6</v>
@@ -238,13 +304,123 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="7">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s" s="7">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C6" t="s" s="3">
         <v>6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="6">
+        <v>14</v>
+      </c>
+      <c r="B7" t="s" s="6">
+        <v>15</v>
+      </c>
+      <c r="C7" t="s" s="4">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="7">
+        <v>16</v>
+      </c>
+      <c r="B8" t="s" s="7">
+        <v>17</v>
+      </c>
+      <c r="C8" t="s" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="6">
+        <v>18</v>
+      </c>
+      <c r="B9" t="s" s="6">
+        <v>19</v>
+      </c>
+      <c r="C9" t="s" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="7">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s" s="7">
+        <v>21</v>
+      </c>
+      <c r="C10" t="s" s="5">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="6">
+        <v>23</v>
+      </c>
+      <c r="B11" t="s" s="6">
+        <v>24</v>
+      </c>
+      <c r="C11" t="s" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="7">
+        <v>25</v>
+      </c>
+      <c r="B12" t="s" s="7">
+        <v>26</v>
+      </c>
+      <c r="C12" t="s" s="4">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="6">
+        <v>27</v>
+      </c>
+      <c r="B13" t="s" s="6">
+        <v>28</v>
+      </c>
+      <c r="C13" t="s" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="7">
+        <v>29</v>
+      </c>
+      <c r="B14" t="s" s="7">
+        <v>30</v>
+      </c>
+      <c r="C14" t="s" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="6">
+        <v>31</v>
+      </c>
+      <c r="B15" t="s" s="6">
+        <v>32</v>
+      </c>
+      <c r="C15" t="s" s="4">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="7">
+        <v>33</v>
+      </c>
+      <c r="B16" t="s" s="7">
+        <v>34</v>
+      </c>
+      <c r="C16" t="s" s="4">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>